<commit_message>
feat: add participant team data spreadsheet
</commit_message>
<xml_diff>
--- a/participants/participant_team.xlsx
+++ b/participants/participant_team.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackcheah/Documents/Personal/mtg-dashboard-v1/participants/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cheah\Documents\MTG-Dashboard\mtg-dashboard-v1\participants\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F09E01E-9C58-7248-A12C-6E59C11A15D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75388BA1-2A61-43D6-B021-0EC019E7CB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17060" yWindow="-23360" windowWidth="36000" windowHeight="22580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14680" yWindow="4360" windowWidth="15980" windowHeight="15590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -241,9 +241,6 @@
     <t>Team RGB</t>
   </si>
   <si>
-    <t>Team Campion</t>
-  </si>
-  <si>
     <t>Team Decay (DKAY)</t>
   </si>
   <si>
@@ -266,6 +263,9 @@
   </si>
   <si>
     <t>Magic Hard to Play</t>
+  </si>
+  <si>
+    <t>2nd Hand Jobs</t>
   </si>
 </sst>
 </file>
@@ -613,13 +613,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -630,7 +630,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -641,7 +641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -652,7 +652,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -663,7 +663,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -674,7 +674,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -685,7 +685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -696,7 +696,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -707,7 +707,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -718,9 +718,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>13</v>
@@ -729,9 +729,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>14</v>
@@ -740,9 +740,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>15</v>
@@ -751,9 +751,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>16</v>
@@ -762,9 +762,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>17</v>
@@ -773,9 +773,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>18</v>
@@ -784,9 +784,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>19</v>
@@ -795,9 +795,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>20</v>
@@ -806,9 +806,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>21</v>
@@ -817,9 +817,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>22</v>
@@ -828,9 +828,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>23</v>
@@ -839,9 +839,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>24</v>
@@ -850,9 +850,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>25</v>
@@ -861,9 +861,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>26</v>
@@ -872,9 +872,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>27</v>
@@ -883,9 +883,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>28</v>
@@ -894,9 +894,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>29</v>
@@ -905,9 +905,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>30</v>
@@ -916,9 +916,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>31</v>
@@ -927,9 +927,9 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>32</v>
@@ -938,9 +938,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>33</v>
@@ -949,9 +949,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>34</v>
@@ -960,9 +960,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>35</v>
@@ -971,9 +971,9 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>36</v>
@@ -982,9 +982,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>37</v>
@@ -993,9 +993,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>38</v>
@@ -1004,9 +1004,9 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>17</v>
@@ -1015,9 +1015,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>39</v>
@@ -1026,9 +1026,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>40</v>
@@ -1037,9 +1037,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>41</v>
@@ -1048,9 +1048,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>42</v>
@@ -1059,9 +1059,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>43</v>
@@ -1070,7 +1070,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>72</v>
       </c>
@@ -1081,7 +1081,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>72</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>72</v>
       </c>
@@ -1103,7 +1103,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>72</v>
       </c>
@@ -1114,9 +1114,9 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>48</v>
@@ -1125,9 +1125,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>49</v>
@@ -1136,9 +1136,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>50</v>
@@ -1147,9 +1147,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>51</v>
@@ -1158,7 +1158,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>71</v>
       </c>
@@ -1169,7 +1169,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>71</v>
       </c>
@@ -1180,7 +1180,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>71</v>
       </c>
@@ -1191,7 +1191,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>71</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>70</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>70</v>
       </c>
@@ -1224,7 +1224,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>70</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>70</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>69</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>69</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>69</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>69</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>68</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>68</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>68</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>68</v>
       </c>

</xml_diff>

<commit_message>
feat: add initial participant team data spreadsheet
</commit_message>
<xml_diff>
--- a/participants/participant_team.xlsx
+++ b/participants/participant_team.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cheah\Documents\MTG-Dashboard\mtg-dashboard-v1\participants\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75388BA1-2A61-43D6-B021-0EC019E7CB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258744C6-9606-4031-9B3F-160805027F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14680" yWindow="4360" windowWidth="15980" windowHeight="15590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19990" yWindow="5080" windowWidth="15980" windowHeight="15590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Teams!$A$1:$C$65</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -46,9 +49,6 @@
     <t>Timothy</t>
   </si>
   <si>
-    <t>Anti Keithing</t>
-  </si>
-  <si>
     <t>Glenn</t>
   </si>
   <si>
@@ -67,9 +67,6 @@
     <t>Jed</t>
   </si>
   <si>
-    <t>Andrew Tiger Boy</t>
-  </si>
-  <si>
     <t>Dom</t>
   </si>
   <si>
@@ -94,21 +91,12 @@
     <t>Hyuk</t>
   </si>
   <si>
-    <t>Vanny</t>
-  </si>
-  <si>
     <t>Ronald</t>
   </si>
   <si>
-    <t>Yi Yang</t>
-  </si>
-  <si>
     <t>Greg</t>
   </si>
   <si>
-    <t>Xavier</t>
-  </si>
-  <si>
     <t>YX</t>
   </si>
   <si>
@@ -151,21 +139,9 @@
     <t>Yun</t>
   </si>
   <si>
-    <t>Derek</t>
-  </si>
-  <si>
     <t>Augustine</t>
   </si>
   <si>
-    <t>silvan</t>
-  </si>
-  <si>
-    <t>ernst</t>
-  </si>
-  <si>
-    <t>sum</t>
-  </si>
-  <si>
     <t>Campion</t>
   </si>
   <si>
@@ -175,18 +151,12 @@
     <t>Yong Xuan</t>
   </si>
   <si>
-    <t>Scott</t>
-  </si>
-  <si>
     <t>Xuan</t>
   </si>
   <si>
     <t>Ivan</t>
   </si>
   <si>
-    <t>wen de</t>
-  </si>
-  <si>
     <t>Yao Yang</t>
   </si>
   <si>
@@ -214,58 +184,91 @@
     <t>Jonathan</t>
   </si>
   <si>
-    <t>de huang</t>
-  </si>
-  <si>
     <t>Yize</t>
   </si>
   <si>
     <t>Cai Jing</t>
   </si>
   <si>
+    <t>Anti Bluefarm Bluefarm Club</t>
+  </si>
+  <si>
+    <t>J Square Sqaured!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snow White and 3 Dwarves </t>
+  </si>
+  <si>
+    <t>有胡须的是你爸爸</t>
+  </si>
+  <si>
+    <t>Team RGB</t>
+  </si>
+  <si>
+    <t>Vengeful Spirit</t>
+  </si>
+  <si>
+    <t>4 Buggers lor</t>
+  </si>
+  <si>
+    <t>Dunman Dogs</t>
+  </si>
+  <si>
+    <t>______goblin deez</t>
+  </si>
+  <si>
+    <t>Team 17</t>
+  </si>
+  <si>
+    <t>Brianstorm</t>
+  </si>
+  <si>
+    <t>Magic Hard to Play</t>
+  </si>
+  <si>
+    <t>2nd Hand Jobs</t>
+  </si>
+  <si>
+    <t>Keith-ers</t>
+  </si>
+  <si>
+    <t>Andrew</t>
+  </si>
+  <si>
+    <t>Silvan</t>
+  </si>
+  <si>
+    <t>Ernst</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t>Een De</t>
+  </si>
+  <si>
+    <t>De Huang</t>
+  </si>
+  <si>
+    <t>Vivian</t>
+  </si>
+  <si>
+    <t>Team Kaya</t>
+  </si>
+  <si>
+    <t>Aron</t>
+  </si>
+  <si>
+    <t>Daryl</t>
+  </si>
+  <si>
+    <t>Ye Yang</t>
+  </si>
+  <si>
+    <t>Xavier Ho</t>
+  </si>
+  <si>
     <t>Vikky</t>
-  </si>
-  <si>
-    <t>Anti Bluefarm Bluefarm Club</t>
-  </si>
-  <si>
-    <t>J Square Sqaured!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Snow White and 3 Dwarves </t>
-  </si>
-  <si>
-    <t>有胡须的是你爸爸</t>
-  </si>
-  <si>
-    <t>Team RGB</t>
-  </si>
-  <si>
-    <t>Team Decay (DKAY)</t>
-  </si>
-  <si>
-    <t>Vengeful Spirit</t>
-  </si>
-  <si>
-    <t>4 Buggers lor</t>
-  </si>
-  <si>
-    <t>Dunman Dogs</t>
-  </si>
-  <si>
-    <t>______goblin deez</t>
-  </si>
-  <si>
-    <t>Team 17</t>
-  </si>
-  <si>
-    <t>Brianstorm</t>
-  </si>
-  <si>
-    <t>Magic Hard to Play</t>
-  </si>
-  <si>
-    <t>2nd Hand Jobs</t>
   </si>
 </sst>
 </file>
@@ -676,10 +679,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -687,10 +690,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -698,10 +701,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -709,10 +712,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9">
         <v>8</v>
@@ -720,10 +723,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -731,10 +734,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -742,10 +745,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>69</v>
       </c>
       <c r="C12">
         <v>11</v>
@@ -753,10 +756,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C13">
         <v>12</v>
@@ -764,10 +767,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14">
         <v>13</v>
@@ -775,10 +778,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C15">
         <v>14</v>
@@ -786,10 +789,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>15</v>
@@ -797,10 +800,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C17">
         <v>16</v>
@@ -808,10 +811,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C18">
         <v>17</v>
@@ -819,10 +822,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C19">
         <v>18</v>
@@ -830,10 +833,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C20">
         <v>19</v>
@@ -841,10 +844,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="C21">
         <v>20</v>
@@ -852,10 +855,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C22">
         <v>21</v>
@@ -863,10 +866,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="C23">
         <v>22</v>
@@ -874,10 +877,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C24">
         <v>23</v>
@@ -885,10 +888,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="C25">
         <v>24</v>
@@ -896,10 +899,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C26">
         <v>25</v>
@@ -907,10 +910,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C27">
         <v>26</v>
@@ -918,10 +921,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C28">
         <v>27</v>
@@ -929,10 +932,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C29">
         <v>28</v>
@@ -940,10 +943,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C30">
         <v>29</v>
@@ -951,10 +954,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C31">
         <v>30</v>
@@ -962,10 +965,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C32">
         <v>31</v>
@@ -973,10 +976,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C33">
         <v>32</v>
@@ -984,10 +987,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C34">
         <v>33</v>
@@ -995,10 +998,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C35">
         <v>34</v>
@@ -1006,10 +1009,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C36">
         <v>35</v>
@@ -1017,10 +1020,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C37">
         <v>36</v>
@@ -1028,10 +1031,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C38">
         <v>37</v>
@@ -1039,10 +1042,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C39">
         <v>38</v>
@@ -1050,10 +1053,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C40">
         <v>39</v>
@@ -1061,10 +1064,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="C41">
         <v>40</v>
@@ -1072,10 +1075,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C42">
         <v>41</v>
@@ -1083,10 +1086,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="C43">
         <v>42</v>
@@ -1094,10 +1097,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>46</v>
+        <v>71</v>
       </c>
       <c r="C44">
         <v>43</v>
@@ -1105,10 +1108,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C45">
         <v>44</v>
@@ -1116,10 +1119,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C46">
         <v>45</v>
@@ -1127,10 +1130,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C47">
         <v>46</v>
@@ -1138,10 +1141,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C48">
         <v>47</v>
@@ -1149,10 +1152,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="C49">
         <v>48</v>
@@ -1160,10 +1163,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C50">
         <v>49</v>
@@ -1171,10 +1174,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C51">
         <v>50</v>
@@ -1182,10 +1185,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="C52">
         <v>51</v>
@@ -1193,10 +1196,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C53">
         <v>52</v>
@@ -1204,10 +1207,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C54">
         <v>53</v>
@@ -1215,10 +1218,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C55">
         <v>54</v>
@@ -1226,10 +1229,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C56">
         <v>55</v>
@@ -1237,10 +1240,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C57">
         <v>56</v>
@@ -1248,10 +1251,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C58">
         <v>57</v>
@@ -1259,10 +1262,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C59">
         <v>58</v>
@@ -1270,10 +1273,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C60">
         <v>59</v>
@@ -1281,10 +1284,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C61">
         <v>60</v>
@@ -1292,10 +1295,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C62">
         <v>61</v>
@@ -1303,10 +1306,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="C63">
         <v>62</v>
@@ -1314,10 +1317,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="C64">
         <v>63</v>
@@ -1325,16 +1328,17 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="C65">
         <v>64</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
UI fix and bug fix: finals not displaying correctly. champion not determined correctly.
</commit_message>
<xml_diff>
--- a/participants/participant_team.xlsx
+++ b/participants/participant_team.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cheah\Documents\MTG-Dashboard\mtg-dashboard-v1\participants\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258744C6-9606-4031-9B3F-160805027F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D95A08-DF40-4FD7-948E-FD8B9DBCC8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19990" yWindow="5080" windowWidth="15980" windowHeight="15590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -244,9 +244,6 @@
     <t>Sum</t>
   </si>
   <si>
-    <t>Een De</t>
-  </si>
-  <si>
     <t>De Huang</t>
   </si>
   <si>
@@ -269,6 +266,9 @@
   </si>
   <si>
     <t>Vikky</t>
+  </si>
+  <si>
+    <t>Wen De</t>
   </si>
 </sst>
 </file>
@@ -847,7 +847,7 @@
         <v>64</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C21">
         <v>20</v>
@@ -869,7 +869,7 @@
         <v>63</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C23">
         <v>22</v>
@@ -891,7 +891,7 @@
         <v>63</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C25">
         <v>24</v>
@@ -1031,7 +1031,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>35</v>
@@ -1042,7 +1042,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>36</v>
@@ -1053,7 +1053,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>37</v>
@@ -1064,10 +1064,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="C41">
         <v>40</v>
@@ -1155,7 +1155,7 @@
         <v>67</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C49">
         <v>48</v>
@@ -1188,7 +1188,7 @@
         <v>58</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C52">
         <v>51</v>
@@ -1298,7 +1298,7 @@
         <v>55</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C62">
         <v>61</v>
@@ -1331,7 +1331,7 @@
         <v>55</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C65">
         <v>64</v>

</xml_diff>

<commit_message>
feat: add end-to-end simulation for 28-team tournament with player drops and ghost verification
</commit_message>
<xml_diff>
--- a/participants/participant_team.xlsx
+++ b/participants/participant_team.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -913,6 +913,1206 @@
         <v>32</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Iota Impact</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Captain_Iota</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Iota Impact</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Scout_Iota</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Iota Impact</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Striker_Iota</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Iota Impact</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Guard_Iota</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Kappa Kings</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Captain_Kappa</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Kappa Kings</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Scout_Kappa</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Kappa Kings</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Striker_Kappa</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Kappa Kings</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Guard_Kappa</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Lambda Legion</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Captain_Lambda</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Lambda Legion</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Scout_Lambda</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Lambda Legion</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Striker_Lambda</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Lambda Legion</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Guard_Lambda</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mu Masters</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Captain_Mu</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Mu Masters</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Scout_Mu</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Mu Masters</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Striker_Mu</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Mu Masters</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Guard_Mu</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Nu Knights</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Captain_Nu</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Nu Knights</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Scout_Nu</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Nu Knights</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Striker_Nu</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Nu Knights</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Guard_Nu</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Xi Xtremes</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Captain_Xi</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Xi Xtremes</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Scout_Xi</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Xi Xtremes</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Striker_Xi</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Xi Xtremes</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Guard_Xi</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Omicron Ops</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Captain_Omicron</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Omicron Ops</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Scout_Omicron</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Omicron Ops</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Striker_Omicron</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Omicron Ops</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Guard_Omicron</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Pi Pioneers</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Captain_Pi</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Pi Pioneers</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Scout_Pi</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Pi Pioneers</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Striker_Pi</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Pi Pioneers</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Guard_Pi</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Rho Raiders</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Captain_Rho</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Rho Raiders</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Scout_Rho</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Rho Raiders</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Striker_Rho</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Rho Raiders</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Guard_Rho</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Sigma Storm</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Captain_Sigma</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Sigma Storm</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Scout_Sigma</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Sigma Storm</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Striker_Sigma</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Sigma Storm</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Guard_Sigma</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Tau Titans</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Captain_Tau</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Tau Titans</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Scout_Tau</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Tau Titans</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Striker_Tau</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Tau Titans</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Guard_Tau</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Upsilon Ultra</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Captain_Upsilon</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Upsilon Ultra</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Scout_Upsilon</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Upsilon Ultra</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Striker_Upsilon</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Upsilon Ultra</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Guard_Upsilon</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Phi Phoenix</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Captain_Phi</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Phi Phoenix</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Scout_Phi</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Phi Phoenix</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Striker_Phi</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Phi Phoenix</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Guard_Phi</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Chi Champions</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Captain_Chi</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Chi Champions</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Scout_Chi</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Chi Champions</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Striker_Chi</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Chi Champions</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Guard_Chi</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Psi Power</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Captain_Psi</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Psi Power</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Scout_Psi</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Psi Power</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Striker_Psi</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Psi Power</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Guard_Psi</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Omega Order</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Captain_Omega</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Omega Order</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Scout_Omega</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Omega Order</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Striker_Omega</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Omega Order</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Guard_Omega</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Atlas Army</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Captain_Atlas</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Atlas Army</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Scout_Atlas</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Atlas Army</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Striker_Atlas</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Atlas Army</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Guard_Atlas</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Bolt Brigade</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Captain_Bolt</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Bolt Brigade</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Scout_Bolt</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Bolt Brigade</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Striker_Bolt</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Bolt Brigade</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Guard_Bolt</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Crux Crew</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Captain_Crux</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Crux Crew</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Scout_Crux</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Crux Crew</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Striker_Crux</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Crux Crew</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Guard_Crux</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Dusk Dynasty</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Captain_Dusk</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Dusk Dynasty</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Scout_Dusk</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Dusk Dynasty</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Striker_Dusk</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Dusk Dynasty</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Guard_Dusk</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>